<commit_message>
Fysik: ljus och ljud som egna kapitel; repetition inför nationella proven som sista kapitel i kemi och fysik
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017mqJrSEX6tzqa8YfkctM6P
</commit_message>
<xml_diff>
--- a/planering/fysik-planering.xlsx
+++ b/planering/fysik-planering.xlsx
@@ -15,10 +15,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Täckning" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Moment'!$A$1:$K$118</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Delområden'!$A$1:$H$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Områden'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Labbar'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Moment'!$A$1:$K$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Delområden'!$A$1:$H$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Områden'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Labbar'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Täckning'!$A$1:$C$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning</t>
+          <t>Ljuskällor och ljusets utbredning</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>ljuskälla, ljusstråle, skugga, ljushastighet</t>
+          <t>ljuskälla, ljusstråle, skugga, ljushastighet, ljusår</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Reflektionslagen; plana speglar; spridd reflektion; färg och ytor.</t>
+          <t>Reflektionslagen; plana speglar; spridd reflektion.</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -3935,17 +3935,17 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Brytning och färger</t>
+          <t>Färg och ytor</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Brytning i vatten och glas; linser och optiska instrument; prisma och ljusets färger.</t>
+          <t>Hur föremål får färg: ljus som absorberas och reflekteras; vitt, svart och färgat ljus.</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>brytning, lins, prisma, spektrum</t>
+          <t>absorption, reflektion, färg, spektrum</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
@@ -3990,17 +3990,17 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Labb: Reflektion och brytning med ljuslåda</t>
+          <t>Labb: Reflektion med ljuslåda</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Hur beter sig ljus vid spegel och i vatten? Eleverna riktar en ljusstråle mot spegel och vattenbehållare, mäter vinklarna och jämför med reflektionslagen. Säkerhet: Titta aldrig in i en laserstråle eller starkt ljus. Rikta inte laser mot ansikten.</t>
+          <t>Hur beter sig ljus när det reflekteras i en spegel? Eleverna riktar en ljusstråle mot en plan spegel, mäter infalls- och reflektionsvinkel och jämför med reflektionslagen. Säkerhet: Titta aldrig in i en laserstråle eller starkt ljus. Rikta inte laser mot ansikten.</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>infallsvinkel, reflektionsvinkel, brytning</t>
+          <t>infallsvinkel, reflektionsvinkel, reflektionslagen</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Optiska instrument: mikroskop och kikare</t>
+          <t>Periskop</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Ögats uppbyggnad</t>
+          <t>Kamouflage och färg</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr"/>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -4115,7 +4115,7 @@
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Fiberoptik</t>
+          <t>Ljusföroreningar</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -4150,17 +4150,17 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Brytning</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Vibrationer; ljud i luft, vätskor och fasta ämnen men inte i vakuum; ljudets hastighet; eko.</t>
+          <t>Ljus mellan luft, vatten och glas; ljusets hastighet i olika medier; totalreflektion.</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>vibration, medium, ljudhastighet, eko</t>
+          <t>brytning, medium, normal, totalreflektion</t>
         </is>
       </c>
       <c r="I78" s="4" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K78" s="4" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -4205,27 +4205,27 @@
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Frekvens, amplitud och hörsel</t>
+          <t>Linser och optiska instrument</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd och frekvens (Hz), ljudstyrka och amplitud (dB); örats funktion; hörselskydd och buller.</t>
+          <t>Konvexa och konkava linser; ögat, kikare, mikroskop och kamera.</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>frekvens, hertz, amplitud, decibel, hörsel</t>
+          <t>lins, brännpunkt, bild, förstoring</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället</t>
+          <t>Kunskaper om fysiken i naturen och samhället; Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -4250,7 +4250,7 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -4260,27 +4260,27 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Registrera ljud</t>
+          <t>Färgspridning och spektrum</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Mikrofon, frekvensanalys och appar; ultraljud och ekolod; ljudisolering.</t>
+          <t>Prisma, regnbåge och ljusets färger.</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>mikrofon, ultraljud, ekolod, ljudisolering</t>
+          <t>prisma, spektrum, regnbåge, färgspridning</t>
         </is>
       </c>
       <c r="I80" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -4315,17 +4315,17 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Labb: Hur påverkar längden tonhöjden?</t>
+          <t>Labb: Brytning i vatten</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras? Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app. Säkerhet: Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
+          <t>Hur bryts ljus när det går från luft till vatten eller glas? Eleverna riktar en ljusstråle mot en halvcylinder av plast eller en vattenbehållare, mäter infalls- och brytningsvinkel och ritar strålgången. Säkerhet: Titta aldrig in i en laserstråle. Torka upp vatten.</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>frekvens, tonhöjd, vibration, app</t>
+          <t>brytningsvinkel, infallsvinkel, medium</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Musikinstrument</t>
+          <t>Fiberoptik</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Dopplereffekten</t>
+          <t>Ögats uppbyggnad</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr"/>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Akustik i klassrummet</t>
+          <t>Optiska instrument i detalj</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr"/>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -4475,17 +4475,17 @@
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Elektromagnetisk strålning</t>
+          <t>Vibrationer och ljudkällor</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>Spektrum från radiovågor till gammastrålning; våglängd och frekvens; synligt ljus, UV och infrarött.</t>
+          <t>Hur ljud uppstår; ljudkällor och vibrerande föremål.</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>spektrum, våglängd, frekvens, UV, infraröd</t>
+          <t>vibration, ljudkälla, svängning</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
@@ -4530,27 +4530,27 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Partikelstrålning och radioaktivitet</t>
+          <t>Ljudets utbredning</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>Alfa-, beta- och gammastrålning; radioaktivt sönderfall och halveringstid; naturlig bakgrundsstrålning.</t>
+          <t>Ljud i luft, vätskor och fasta ämnen men inte i vakuum; ljudets hastighet.</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>radioaktivitet, halveringstid, alfa, beta, gamma</t>
+          <t>medium, ljudhastighet, vakuum</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället</t>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -4585,32 +4585,32 @@
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Användning och risker</t>
+          <t>Eko och ljudisolering</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Röntgen, mikrovågsugn, solljus, mobiler och kärnkraft: nytta, risker och skydd; granskning av påståenden.</t>
+          <t>Reflektion och absorption av ljud; eko, efterklang och ljudisolering.</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>röntgen, strålskydd, solskydd, risk</t>
+          <t>eko, absorption, ljudisolering</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>Formulera egna och granska andras argument; kommunicera; hantera praktiska och etiska valsituationer om energi, teknik och miljö; Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
+          <t>Kunskaper om fysiken i naturen och samhället</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker; Informationssökning, kritisk granskning och användning av information som rör fysik</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
         <is>
-          <t>Granska information, kommunicera och ta ställning</t>
+          <t>Begrepp och förklaringsmodeller</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -4640,17 +4640,17 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Labb: Vad stoppar UV-strålning?</t>
+          <t>Labb: Hur snabbt går ljudet?</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>Vilka material och solskyddsfaktorer skyddar mot UV-strålning? Eleverna använder UV-känsliga pärlor under UV-lampa eller solljus, täcker med olika material och solkräm och jämför färgförändringen. Säkerhet: Titta inte rakt in i UV-lampan. Använd solkräm enligt märkning och tvätta händerna.</t>
+          <t>Hur kan ljudets hastighet mätas? Eleverna mäter tid för eko över en känd sträcka eller med två mikrofoner och en app, och beräknar v = s/t. Säkerhet: Skydda hörseln: inga höga smällar. Håll avstånd vid utomhusmätning.</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>UV-strålning, skydd, solskyddsfaktor</t>
+          <t>ljudhastighet, sträcka, tid, eko</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K88" s="4" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Röntgen i sjukvården</t>
+          <t>Åska och ljudets hastighet</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr"/>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Kärnkraft och avfall</t>
+          <t>Överljud</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr"/>
@@ -4745,7 +4745,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Strålning från mobiler</t>
+          <t>Ljud under vatten</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -4800,17 +4800,17 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Jordens strålningsbalans</t>
+          <t>Frekvens och amplitud</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Solinstrålning, albedo, reflektion och utstrålning; varför jorden håller en jämn temperatur.</t>
+          <t>Tonhöjd och frekvens (Hz), ljudstyrka och amplitud (dB).</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>solstrålning, albedo, utstrålning, balans</t>
+          <t>frekvens, hertz, amplitud, decibel</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
-          <t>Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -4855,27 +4855,27 @@
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Växthuseffekten</t>
+          <t>Hörsel och hörselskydd</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Naturlig växthuseffekt; växthusgaser och deras källor; förstärkt växthuseffekt.</t>
+          <t>Örats funktion; buller och hörselskador; hörselskydd.</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>växthusgas, växthuseffekt, infraröd strålning</t>
+          <t>örat, buller, hörselskada, hörselskydd</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+          <t>Kunskaper om fysiken i naturen och samhället</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
-          <t>Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -4910,32 +4910,32 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Klimatförändringar och ställningstagande</t>
+          <t>Registrera ljud</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Klimatdata och modeller; orsaker, konsekvenser och åtgärder; granska information om klimat.</t>
+          <t>Mikrofon, frekvensanalys och appar; ultraljud och ekolod.</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>klimatmodell, prognos, åtgärd, källkritik</t>
+          <t>mikrofon, ultraljud, ekolod, frekvensanalys</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>Formulera egna och granska andras argument; kommunicera; hantera praktiska och etiska valsituationer om energi, teknik och miljö; Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
+          <t>Kunskaper om fysiken i naturen och samhället; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar; Informationssökning, kritisk granskning och användning av information som rör fysik; Argumentation och ställningstaganden i aktuella frågor som rör energi, teknik och miljö</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
         <is>
-          <t>Granska information, kommunicera och ta ställning</t>
+          <t>Begrepp och förklaringsmodeller</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -4965,17 +4965,17 @@
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Labb: Hur påverkar ytans färg uppvärmningen?</t>
+          <t>Labb: Hur påverkar längden tonhöjden?</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>Hur påverkar ytans färg temperaturen när den belyses? Eleverna belyser svarta, vita och silverfärgade ytor med lampa och mäter temperaturen över tid. De kopplar till albedo och klimat. Säkerhet: Lampan blir varm. Rör inte lampa eller glödande delar.</t>
+          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras? Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden, eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app. Säkerhet: Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>albedo, absorption, reflektion, temperatur</t>
+          <t>frekvens, tonhöjd, vibration, app</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K95" s="4" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Istider och klimatets historia</t>
+          <t>Musikinstrument</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr"/>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Ozonskiktet</t>
+          <t>Dopplereffekten</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr"/>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Havens roll i klimatet</t>
+          <t>Akustik i klassrummet</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -5105,7 +5105,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
@@ -5125,17 +5125,17 @@
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>Solsystemet och gravitation</t>
+          <t>Elektromagnetisk strålning</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>Solen, planeterna och deras banor; gravitation; månens faser; avstånd i solsystemet.</t>
+          <t>Spektrum från radiovågor till gammastrålning; våglängd och frekvens; synligt ljus, UV och infrarött.</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>gravitation, planet, bana, ljusminut</t>
+          <t>spektrum, våglängd, frekvens, UV, infraröd</t>
         </is>
       </c>
       <c r="I99" s="4" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="J99" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Krafter, rörelser och rörelseförändringar och hur kunskaper om detta används, t.ex. i frågor om trafiksäkerhet</t>
+          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
         </is>
       </c>
       <c r="K99" s="4" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
@@ -5180,17 +5180,17 @@
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Stjärnor och galaxer</t>
+          <t>Partikelstrålning och radioaktivitet</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>Stjärnors livscykel, Vintergatan och galaxer; ljusår och avstånd.</t>
+          <t>Alfa-, beta- och gammastrålning; radioaktivt sönderfall och halveringstid; naturlig bakgrundsstrålning.</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr">
         <is>
-          <t>stjärna, galax, ljusår, livscykel</t>
+          <t>radioaktivitet, halveringstid, alfa, beta, gamma</t>
         </is>
       </c>
       <c r="I100" s="4" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J100" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
         </is>
       </c>
       <c r="K100" s="4" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
@@ -5235,32 +5235,32 @@
       </c>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Big bang och universums utveckling</t>
+          <t>Användning och risker</t>
         </is>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>Expansion, rödförskjutning och bakgrundsstrålning; hur modellen vuxit fram och ändrats.</t>
+          <t>Röntgen, mikrovågsugn, solljus, mobiler och kärnkraft: nytta, risker och skydd; granskning av påståenden.</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>big bang, expansion, rödförskjutning</t>
+          <t>röntgen, strålskydd, solskydd, risk</t>
         </is>
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen; Skilja mellan naturvetenskapliga och andra sätt att beskriva och förklara omvärlden</t>
+          <t>Formulera egna och granska andras argument; kommunicera; hantera praktiska och etiska valsituationer om energi, teknik och miljö; Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Sambandet mellan undersökningar och begrepp och förklaringsmodeller; modellernas historiska framväxt, användbarhet och föränderlighet</t>
+          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker; Informationssökning, kritisk granskning och användning av information som rör fysik</t>
         </is>
       </c>
       <c r="K101" s="4" t="inlineStr">
         <is>
-          <t>Begrepp och förklaringsmodeller</t>
+          <t>Granska information, kommunicera och ta ställning</t>
         </is>
       </c>
     </row>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
@@ -5290,32 +5290,32 @@
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Labb: Solsystemet i skala</t>
+          <t>Labb: Vad stoppar UV-strålning?</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>Hur stort är solsystemet jämfört med planeterna? Eleverna bygger en skalmodell med beräknade avstånd (t.ex. 1 m = 1 AU) och diskuterar vad modellen visar och inte visar. Säkerhet: Inga särskilda risker.</t>
+          <t>Vilka material och solskyddsfaktorer skyddar mot UV-strålning? Eleverna använder UV-känsliga pärlor under UV-lampa eller solljus, täcker med olika material och solkräm och jämför färgförändringen. Säkerhet: Titta inte rakt in i UV-lampan. Använd solkräm enligt märkning och tvätta händerna.</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr">
         <is>
-          <t>skala, avstånd, modell, begränsning</t>
+          <t>UV-strålning, skydd, solskyddsfaktor</t>
         </is>
       </c>
       <c r="I102" s="4" t="inlineStr">
         <is>
-          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
+          <t>Egna systematiska undersökningar: påståenden kan prövas och kunskap växer fram med naturvetenskapliga arbetsmetoder; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
         </is>
       </c>
       <c r="J102" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
         </is>
       </c>
       <c r="K102" s="4" t="inlineStr">
         <is>
-          <t>Begrepp och förklaringsmodeller; Systematiska undersökningar</t>
+          <t>Systematiska undersökningar</t>
         </is>
       </c>
     </row>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E103" s="4" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Svarta hål</t>
+          <t>Röntgen i sjukvården</t>
         </is>
       </c>
       <c r="G103" s="4" t="inlineStr"/>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Rymdteleskop</t>
+          <t>Kärnkraft och avfall</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr"/>
@@ -5395,7 +5395,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>Rymdfärder</t>
+          <t>Strålning från mobiler</t>
         </is>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
@@ -5450,27 +5450,27 @@
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>Exoplaneter och hur vi hittar dem</t>
+          <t>Jordens strålningsbalans</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>Transitmetoden och radialhastighet; vad mätdata säger om planeternas storlek och bana.</t>
+          <t>Solinstrålning, albedo, reflektion och utstrålning; varför jorden håller en jämn temperatur.</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
         <is>
-          <t>exoplanet, transit, ljuskurva</t>
+          <t>solstrålning, albedo, utstrålning, balans</t>
         </is>
       </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället</t>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J106" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+          <t>Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar</t>
         </is>
       </c>
       <c r="K106" s="4" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E107" s="4" t="inlineStr">
@@ -5505,17 +5505,17 @@
       </c>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>Livets villkor och beboeliga zonen</t>
+          <t>Växthuseffekten</t>
         </is>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>Vatten, temperatur, atmosfär och energikälla; den beboeliga zonen; livet på jorden som jämförelse.</t>
+          <t>Naturlig växthuseffekt; växthusgaser och deras källor; förstärkt växthuseffekt.</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>beboelig zon, atmosfär, flytande vatten</t>
+          <t>växthusgas, växthuseffekt, infraröd strålning</t>
         </is>
       </c>
       <c r="I107" s="4" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="J107" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+          <t>Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar</t>
         </is>
       </c>
       <c r="K107" s="4" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
@@ -5560,27 +5560,27 @@
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>Granska rymdnyheter</t>
+          <t>Klimatförändringar och ställningstagande</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>Hur vet vi? Källor, rubriker och belägg; skillnad mellan hypotes och bevis.</t>
+          <t>Klimatdata och modeller; orsaker, konsekvenser och åtgärder; granska information om klimat.</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
         <is>
-          <t>hypotes, belägg, källkritik, rubrik</t>
+          <t>klimatmodell, prognos, åtgärd, källkritik</t>
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
-          <t>Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
+          <t>Formulera egna och granska andras argument; kommunicera; hantera praktiska och etiska valsituationer om energi, teknik och miljö; Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
         </is>
       </c>
       <c r="J108" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Informationssökning, kritisk granskning och användning av information som rör fysik; Argumentation och ställningstaganden i aktuella frågor som rör energi, teknik och miljö</t>
+          <t>Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar; Informationssökning, kritisk granskning och användning av information som rör fysik; Argumentation och ställningstaganden i aktuella frågor som rör energi, teknik och miljö</t>
         </is>
       </c>
       <c r="K108" s="4" t="inlineStr">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
@@ -5615,17 +5615,17 @@
       </c>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>Labb: Transitmetoden: hur upptäcks planeter?</t>
+          <t>Labb: Hur påverkar ytans färg uppvärmningen?</t>
         </is>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>Hur ändras ljusstyrkan när en planet passerar framför sin stjärna? Eleverna låter en liten boll kretsa framför en lampa och mäter ljusstyrkan med app. De ritar ljuskurvan och kopplar till planetens storlek. Säkerhet: Lampan blir varm. Tänd bara när det behövs.</t>
+          <t>Hur påverkar ytans färg temperaturen när den belyses? Eleverna belyser svarta, vita och silverfärgade ytor med lampa och mäter temperaturen över tid. De kopplar till albedo och klimat. Säkerhet: Lampan blir varm. Rör inte lampa eller glödande delar.</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>transit, ljuskurva, ljusstyrka</t>
+          <t>albedo, absorption, reflektion, temperatur</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="J109" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar</t>
         </is>
       </c>
       <c r="K109" s="4" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>Mars och livet</t>
+          <t>Istider och klimatets historia</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr"/>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>Drake-ekvationen</t>
+          <t>Ozonskiktet</t>
         </is>
       </c>
       <c r="G111" s="4" t="inlineStr"/>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>SETI</t>
+          <t>Havens roll i klimatet</t>
         </is>
       </c>
       <c r="G112" s="4" t="inlineStr"/>
@@ -5751,21 +5751,21 @@
     </row>
     <row r="113">
       <c r="A113" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Repetition inför nationella proven</t>
+          <t>Universums uppkomst och uppbyggnad</t>
         </is>
       </c>
       <c r="E113" s="4" t="inlineStr">
@@ -5775,17 +5775,17 @@
       </c>
       <c r="F113" s="4" t="inlineStr">
         <is>
-          <t>Repetition: partikelmodell, energi och krafter</t>
+          <t>Solsystemet och gravitation</t>
         </is>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>Samlad repetition av partikelmodell, tryck och densitet, energi och krafter med övningsuppgifter från tidigare nationella prov.</t>
+          <t>Solen, planeterna och deras banor; gravitation; månens faser; avstånd i solsystemet.</t>
         </is>
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>partikel, energi, kraft, tryck, densitet</t>
+          <t>gravitation, planet, bana, ljusminut</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="J113" s="4" t="inlineStr">
         <is>
-          <t>Partikelmodell av materiens egenskaper samt fasövergångar, tryck, volym, densitet och temperatur; Energins flöde och oförstörbarhet samt energislags kvalitet; energikällor och deras för- och nackdelar för samhället och miljön; Krafter, rörelser och rörelseförändringar och hur kunskaper om detta används, t.ex. i frågor om trafiksäkerhet</t>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Krafter, rörelser och rörelseförändringar och hur kunskaper om detta används, t.ex. i frågor om trafiksäkerhet</t>
         </is>
       </c>
       <c r="K113" s="4" t="inlineStr">
@@ -5806,21 +5806,21 @@
     </row>
     <row r="114">
       <c r="A114" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Repetition inför nationella proven</t>
+          <t>Universums uppkomst och uppbyggnad</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
@@ -5830,27 +5830,27 @@
       </c>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>Repetition: elektricitet, ljus, ljud och strålning</t>
+          <t>Stjärnor och galaxer</t>
         </is>
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
-          <t>Samlad repetition av kretsar, magnetism, ljus, ljud och strålning.</t>
+          <t>Stjärnors livscykel, Vintergatan och galaxer; ljusår och avstånd.</t>
         </is>
       </c>
       <c r="H114" s="4" t="inlineStr">
         <is>
-          <t>krets, magnetfält, ljus, ljud, strålning</t>
+          <t>stjärna, galax, ljusår, livscykel</t>
         </is>
       </c>
       <c r="I114" s="4" t="inlineStr">
         <is>
-          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+          <t>Kunskaper om fysiken i naturen och samhället</t>
         </is>
       </c>
       <c r="J114" s="4" t="inlineStr">
         <is>
-          <t>Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker; Hur ljus breder ut sig, reflekteras och bryts; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt; Sambandet mellan elektricitet och magnetism samt mellan ström och spänning i elektriska kretsar; kretsar i elektrisk utrustning</t>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
         </is>
       </c>
       <c r="K114" s="4" t="inlineStr">
@@ -5861,21 +5861,21 @@
     </row>
     <row r="115">
       <c r="A115" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>Repetition inför nationella proven</t>
+          <t>Universums uppkomst och uppbyggnad</t>
         </is>
       </c>
       <c r="E115" s="4" t="inlineStr">
@@ -5885,87 +5885,107 @@
       </c>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>Repetition: undersökningar och argument</t>
+          <t>Big bang och universums utveckling</t>
         </is>
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
-          <t>Planera och värdera undersökningar, tolka diagram, granska källor och argumentera om energi, teknik och miljö.</t>
+          <t>Expansion, rödförskjutning och bakgrundsstrålning; hur modellen vuxit fram och ändrats.</t>
         </is>
       </c>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>variabel, diagram, källkritik, argument</t>
+          <t>big bang, expansion, rödförskjutning</t>
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>Formulera egna och granska andras argument; kommunicera; hantera praktiska och etiska valsituationer om energi, teknik och miljö</t>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen; Skilja mellan naturvetenskapliga och andra sätt att beskriva och förklara omvärlden</t>
         </is>
       </c>
       <c r="J115" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Sambandet mellan undersökningar och begrepp och förklaringsmodeller; modellernas historiska framväxt, användbarhet och föränderlighet; Informationssökning, kritisk granskning och användning av information som rör fysik; Argumentation och ställningstaganden i aktuella frågor som rör energi, teknik och miljö</t>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Sambandet mellan undersökningar och begrepp och förklaringsmodeller; modellernas historiska framväxt, användbarhet och föränderlighet</t>
         </is>
       </c>
       <c r="K115" s="4" t="inlineStr">
         <is>
-          <t>Granska information, kommunicera och ta ställning; Systematiska undersökningar</t>
+          <t>Begrepp och förklaringsmodeller</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>Repetition inför nationella proven</t>
+          <t>Universums uppkomst och uppbyggnad</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>Om tid / fördjupning</t>
+          <t>Labb</t>
         </is>
       </c>
       <c r="F116" s="4" t="inlineStr">
         <is>
-          <t>Gamla nationella prov</t>
-        </is>
-      </c>
-      <c r="G116" s="4" t="inlineStr"/>
-      <c r="H116" s="4" t="inlineStr"/>
-      <c r="I116" s="4" t="inlineStr"/>
-      <c r="J116" s="4" t="inlineStr"/>
-      <c r="K116" s="4" t="inlineStr"/>
+          <t>Labb: Solsystemet i skala</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>Hur stort är solsystemet jämfört med planeterna? Eleverna bygger en skalmodell med beräknade avstånd (t.ex. 1 m = 1 AU) och diskuterar vad modellen visar och inte visar. Säkerhet: Inga särskilda risker.</t>
+        </is>
+      </c>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>skala, avstånd, modell, begränsning</t>
+        </is>
+      </c>
+      <c r="I116" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
+        </is>
+      </c>
+      <c r="J116" s="4" t="inlineStr">
+        <is>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="K116" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller; Systematiska undersökningar</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>Repetition inför nationella proven</t>
+          <t>Universums uppkomst och uppbyggnad</t>
         </is>
       </c>
       <c r="E117" s="4" t="inlineStr">
@@ -5975,7 +5995,7 @@
       </c>
       <c r="F117" s="4" t="inlineStr">
         <is>
-          <t>Provstrategier</t>
+          <t>Svarta hål</t>
         </is>
       </c>
       <c r="G117" s="4" t="inlineStr"/>
@@ -5986,21 +6006,21 @@
     </row>
     <row r="118">
       <c r="A118" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>Repetition inför nationella proven</t>
+          <t>Universums uppkomst och uppbyggnad</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
@@ -6010,7 +6030,7 @@
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>Begreppskartor</t>
+          <t>Rymdteleskop</t>
         </is>
       </c>
       <c r="G118" s="4" t="inlineStr"/>
@@ -6019,8 +6039,1034 @@
       <c r="J118" s="4" t="inlineStr"/>
       <c r="K118" s="4" t="inlineStr"/>
     </row>
+    <row r="119">
+      <c r="A119" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Universums uppkomst och uppbyggnad</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>Rymdfärder</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr"/>
+      <c r="H119" s="4" t="inlineStr"/>
+      <c r="I119" s="4" t="inlineStr"/>
+      <c r="J119" s="4" t="inlineStr"/>
+      <c r="K119" s="4" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>Exoplaneter och hur vi hittar dem</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>Transitmetoden och radialhastighet; vad mätdata säger om planeternas storlek och bana.</t>
+        </is>
+      </c>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>exoplanet, transit, ljuskurva</t>
+        </is>
+      </c>
+      <c r="I120" s="4" t="inlineStr">
+        <is>
+          <t>Kunskaper om fysiken i naturen och samhället</t>
+        </is>
+      </c>
+      <c r="J120" s="4" t="inlineStr">
+        <is>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="K120" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>Livets villkor och beboeliga zonen</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>Vatten, temperatur, atmosfär och energikälla; den beboeliga zonen; livet på jorden som jämförelse.</t>
+        </is>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>beboelig zon, atmosfär, flytande vatten</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J121" s="4" t="inlineStr">
+        <is>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="K121" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>Granska rymdnyheter</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>Hur vet vi? Källor, rubriker och belägg; skillnad mellan hypotes och bevis.</t>
+        </is>
+      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>hypotes, belägg, källkritik, rubrik</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="inlineStr">
+        <is>
+          <t>Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
+        </is>
+      </c>
+      <c r="J122" s="4" t="inlineStr">
+        <is>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Informationssökning, kritisk granskning och användning av information som rör fysik; Argumentation och ställningstaganden i aktuella frågor som rör energi, teknik och miljö</t>
+        </is>
+      </c>
+      <c r="K122" s="4" t="inlineStr">
+        <is>
+          <t>Granska information, kommunicera och ta ställning</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>Labb</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>Labb: Transitmetoden: hur upptäcks planeter?</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>Hur ändras ljusstyrkan när en planet passerar framför sin stjärna? Eleverna låter en liten boll kretsa framför en lampa och mäter ljusstyrkan med app. De ritar ljuskurvan och kopplar till planetens storlek. Säkerhet: Lampan blir varm. Tänd bara när det behövs.</t>
+        </is>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>transit, ljuskurva, ljusstyrka</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>Egna systematiska undersökningar: påståenden kan prövas och kunskap växer fram med naturvetenskapliga arbetsmetoder; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="inlineStr">
+        <is>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="K123" s="4" t="inlineStr">
+        <is>
+          <t>Systematiska undersökningar</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>Mars och livet</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr"/>
+      <c r="H124" s="4" t="inlineStr"/>
+      <c r="I124" s="4" t="inlineStr"/>
+      <c r="J124" s="4" t="inlineStr"/>
+      <c r="K124" s="4" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>Drake-ekvationen</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr"/>
+      <c r="H125" s="4" t="inlineStr"/>
+      <c r="I125" s="4" t="inlineStr"/>
+      <c r="J125" s="4" t="inlineStr"/>
+      <c r="K125" s="4" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>SETI</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr"/>
+      <c r="H126" s="4" t="inlineStr"/>
+      <c r="I126" s="4" t="inlineStr"/>
+      <c r="J126" s="4" t="inlineStr"/>
+      <c r="K126" s="4" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Materia, energi och krafter</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>Partikelmodell, tryck och densitet: repetition</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>Partikelmodellen, fasövergångar, tryck, volym, densitet och temperatur; enkla beräkningar.</t>
+        </is>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>partikel, tryck, densitet, fasövergång</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J127" s="4" t="inlineStr">
+        <is>
+          <t>Partikelmodell av materiens egenskaper samt fasövergångar, tryck, volym, densitet och temperatur</t>
+        </is>
+      </c>
+      <c r="K127" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>Materia, energi och krafter</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>Energi och energikällor: repetition</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>Energiomvandlingar, energins oförstörbarhet och kvalitet; energikällors för- och nackdelar.</t>
+        </is>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>energiform, verkningsgrad, energikälla</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr">
+        <is>
+          <t>Energins flöde och oförstörbarhet samt energislags kvalitet; energikällor och deras för- och nackdelar för samhället och miljön</t>
+        </is>
+      </c>
+      <c r="K128" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>Materia, energi och krafter</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>Krafter och rörelse: repetition</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>Krafter, Newtons lagar, hastighet och trafiksäkerhet; enkla beräkningar.</t>
+        </is>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>kraft, hastighet, acceleration, bromssträcka</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J129" s="4" t="inlineStr">
+        <is>
+          <t>Krafter, rörelser och rörelseförändringar och hur kunskaper om detta används, t.ex. i frågor om trafiksäkerhet</t>
+        </is>
+      </c>
+      <c r="K129" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>Materia, energi och krafter</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>Gamla nationella prov</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr"/>
+      <c r="H130" s="4" t="inlineStr"/>
+      <c r="I130" s="4" t="inlineStr"/>
+      <c r="J130" s="4" t="inlineStr"/>
+      <c r="K130" s="4" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>Materia, energi och krafter</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
+          <t>Begreppskartor</t>
+        </is>
+      </c>
+      <c r="G131" s="4" t="inlineStr"/>
+      <c r="H131" s="4" t="inlineStr"/>
+      <c r="I131" s="4" t="inlineStr"/>
+      <c r="J131" s="4" t="inlineStr"/>
+      <c r="K131" s="4" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>Elektricitet, ljus, ljud, strålning och universum</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>Elektricitet och magnetism: repetition</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>Kretsar, ström och spänning, elektromagnetism.</t>
+        </is>
+      </c>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>krets, ström, spänning, elektromagnet</t>
+        </is>
+      </c>
+      <c r="I132" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J132" s="4" t="inlineStr">
+        <is>
+          <t>Sambandet mellan elektricitet och magnetism samt mellan ström och spänning i elektriska kretsar; kretsar i elektrisk utrustning</t>
+        </is>
+      </c>
+      <c r="K132" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>Elektricitet, ljus, ljud, strålning och universum</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>Ljus och ljud: repetition</t>
+        </is>
+      </c>
+      <c r="G133" s="4" t="inlineStr">
+        <is>
+          <t>Reflektion, brytning, ljudets uppkomst och utbredning.</t>
+        </is>
+      </c>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>reflektion, brytning, vibration, frekvens</t>
+        </is>
+      </c>
+      <c r="I133" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J133" s="4" t="inlineStr">
+        <is>
+          <t>Hur ljus breder ut sig, reflekteras och bryts; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+        </is>
+      </c>
+      <c r="K133" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>Elektricitet, ljus, ljud, strålning och universum</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>Strålning, klimat och universum: repetition</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>Strålning, strålningsbalans och växthuseffekt; universums uppbyggnad.</t>
+        </is>
+      </c>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>strålning, växthuseffekt, universum</t>
+        </is>
+      </c>
+      <c r="I134" s="4" t="inlineStr">
+        <is>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+        </is>
+      </c>
+      <c r="J134" s="4" t="inlineStr">
+        <is>
+          <t>Universums uppkomst, uppbyggnad och utveckling samt förutsättningar för att finna planeter och liv i andra solsystem; Fysikaliska förklaringsmodeller av jordens strålningsbalans, växthuseffekten och klimatförändringar; Partikelstrålning och elektromagnetisk strålning, deras användningsområden och risker</t>
+        </is>
+      </c>
+      <c r="K134" s="4" t="inlineStr">
+        <is>
+          <t>Begrepp och förklaringsmodeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>Elektricitet, ljus, ljud, strålning och universum</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>Gamla nationella prov</t>
+        </is>
+      </c>
+      <c r="G135" s="4" t="inlineStr"/>
+      <c r="H135" s="4" t="inlineStr"/>
+      <c r="I135" s="4" t="inlineStr"/>
+      <c r="J135" s="4" t="inlineStr"/>
+      <c r="K135" s="4" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>Undersökningar, källor och argument</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>Planera och värdera undersökningar</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>Variabler, rättvist försök, mätfel; läsa tabeller och diagram.</t>
+        </is>
+      </c>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>variabel, felkälla, tabell, diagram</t>
+        </is>
+      </c>
+      <c r="I136" s="4" t="inlineStr"/>
+      <c r="J136" s="4" t="inlineStr">
+        <is>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Sambandet mellan undersökningar och begrepp och förklaringsmodeller; modellernas historiska framväxt, användbarhet och föränderlighet</t>
+        </is>
+      </c>
+      <c r="K136" s="4" t="inlineStr">
+        <is>
+          <t>Systematiska undersökningar</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>Undersökningar, källor och argument</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>Granska källor</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>Källor, avsändare och syfte; fysikpåståenden i media.</t>
+        </is>
+      </c>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>källa, trovärdighet, påstående</t>
+        </is>
+      </c>
+      <c r="I137" s="4" t="inlineStr">
+        <is>
+          <t>Söka svar på ämnesspecifika frågor med olika typer av källor; kritiskt tänkande</t>
+        </is>
+      </c>
+      <c r="J137" s="4" t="inlineStr">
+        <is>
+          <t>Informationssökning, kritisk granskning och användning av information som rör fysik</t>
+        </is>
+      </c>
+      <c r="K137" s="4" t="inlineStr">
+        <is>
+          <t>Granska information, kommunicera och ta ställning</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>Undersökningar, källor och argument</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>Lektionsmoment</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>Argumentera om energi, teknik och miljö</t>
+        </is>
+      </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>Argumentera med belägg och motargument.</t>
+        </is>
+      </c>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>argument, belägg, motargument</t>
+        </is>
+      </c>
+      <c r="I138" s="4" t="inlineStr">
+        <is>
+          <t>Formulera egna och granska andras argument; kommunicera; hantera praktiska och etiska valsituationer om energi, teknik och miljö</t>
+        </is>
+      </c>
+      <c r="J138" s="4" t="inlineStr">
+        <is>
+          <t>Argumentation och ställningstaganden i aktuella frågor som rör energi, teknik och miljö</t>
+        </is>
+      </c>
+      <c r="K138" s="4" t="inlineStr">
+        <is>
+          <t>Granska information, kommunicera och ta ställning</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>Undersökningar, källor och argument</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="inlineStr">
+        <is>
+          <t>Gamla nationella prov</t>
+        </is>
+      </c>
+      <c r="G139" s="4" t="inlineStr"/>
+      <c r="H139" s="4" t="inlineStr"/>
+      <c r="I139" s="4" t="inlineStr"/>
+      <c r="J139" s="4" t="inlineStr"/>
+      <c r="K139" s="4" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>Undersökningar, källor och argument</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="inlineStr">
+        <is>
+          <t>Om tid / fördjupning</t>
+        </is>
+      </c>
+      <c r="F140" s="4" t="inlineStr">
+        <is>
+          <t>Provstrategier</t>
+        </is>
+      </c>
+      <c r="G140" s="4" t="inlineStr"/>
+      <c r="H140" s="4" t="inlineStr"/>
+      <c r="I140" s="4" t="inlineStr"/>
+      <c r="J140" s="4" t="inlineStr"/>
+      <c r="K140" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K118"/>
+  <autoFilter ref="A1:K140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6031,7 +7077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6492,7 +7538,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -6502,17 +7548,17 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara och rita hur ljus breder ut sig, reflekteras och bryts och ge exempel på optiska instrument.</t>
+          <t>Eleven kan förklara och rita hur ljus breder ut sig och reflekteras och förklara skuggor, speglar och färg.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver ljusets utbredning och ger exempel på reflektion och brytning. C: ritar strålgångar och förklarar skuggor, speglar och linser. A: förklarar och förutsäger brytning och färgspridning.</t>
+          <t>E: beskriver ljusets utbredning och ger exempel på reflektion. C: ritar strålgångar och förklarar skuggor och speglar. A: förklarar och förutsäger reflektion och hur ytor ger färg.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -6522,7 +7568,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Optiska instrument: mikroskop och kikare; Ögats uppbyggnad; Fiberoptik</t>
+          <t>Periskop; Kamouflage och färg; Ljusföroreningar</t>
         </is>
       </c>
     </row>
@@ -6532,7 +7578,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -6542,27 +7588,27 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara hur ljud uppstår, breder ut sig och registreras och hur hörseln kan skyddas.</t>
+          <t>Eleven kan förklara och rita brytning av ljus och hur linser och optiska instrument fungerar.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver att ljud är vibrationer och ger exempel. C: förklarar frekvens, amplitud och ljudets utbredning. A: resonerar om mätvärden, hörselskador och registrering med digitala verktyg.</t>
+          <t>E: beskriver brytning och ger exempel. C: ritar strålgångar genom linser och förklarar prismat. A: förklarar och förutsäger brytning och färgspridning.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Vågmodell</t>
+          <t>Ljusstrålemodell</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Musikinstrument; Dopplereffekten; Akustik i klassrummet</t>
+          <t>Fiberoptik; Ögats uppbyggnad; Optiska instrument i detalj</t>
         </is>
       </c>
     </row>
@@ -6572,7 +7618,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -6582,27 +7628,27 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan skilja mellan partikelstrålning och elektromagnetisk strålning och beskriva användning och risker.</t>
+          <t>Eleven kan förklara att ljud är vibrationer som breder ut sig i ett medium och beräkna ljudets hastighet.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>E: ger exempel på strålning och nytta och risk. C: förklarar skillnader och skyddsåtgärder. A: väger nytta mot risk i aktuella frågor och motiverar med källor.</t>
+          <t>E: beskriver att ljud är vibrationer och ger exempel. C: förklarar utbredning i olika medier och beräknar hastighet. A: resonerar om mätvärden och om hur ljud reflekteras och absorberas.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Strålningsmodell</t>
+          <t>Vågmodell</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Röntgen i sjukvården; Kärnkraft och avfall; Strålning från mobiler</t>
+          <t>Åska och ljudets hastighet; Överljud; Ljud under vatten</t>
         </is>
       </c>
     </row>
@@ -6612,7 +7658,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -6622,27 +7668,27 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara jordens strålningsbalans och växthuseffekten och argumentera om klimatförändringar med belägg.</t>
+          <t>Eleven kan förklara frekvens och amplitud, hur hörseln fungerar och hur ljud registreras.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver växthuseffekten och ger exempel på klimatpåverkan. C: förklarar strålningsbalansen och skillnaden mellan naturlig och förstärkt effekt. A: bedömer klimatmodeller och åtgärder med belägg från flera källor.</t>
+          <t>E: beskriver tonhöjd, ljudstyrka och hörselskydd. C: förklarar frekvens, amplitud och örats funktion. A: resonerar om mätvärden, hörselskador och registrering med digitala verktyg.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalansmodell</t>
+          <t>Vågmodell</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Istider och klimatets historia; Ozonskiktet; Havens roll i klimatet</t>
+          <t>Musikinstrument; Dopplereffekten; Akustik i klassrummet</t>
         </is>
       </c>
     </row>
@@ -6652,7 +7698,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -6662,27 +7708,27 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan beskriva universums uppbyggnad och utveckling och förklara hur modellerna vuxit fram.</t>
+          <t>Eleven kan skilja mellan partikelstrålning och elektromagnetisk strålning och beskriva användning och risker.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver solsystem, galaxer och big bang. C: förklarar bevisen för ett expanderande universum. A: resonerar om modellernas styrkor, begränsningar och föränderlighet.</t>
+          <t>E: ger exempel på strålning och nytta och risk. C: förklarar skillnader och skyddsåtgärder. A: väger nytta mot risk i aktuella frågor och motiverar med källor.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Universummodell</t>
+          <t>Strålningsmodell</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Svarta hål; Rymdteleskop; Rymdfärder</t>
+          <t>Röntgen i sjukvården; Kärnkraft och avfall; Strålning från mobiler</t>
         </is>
       </c>
     </row>
@@ -6692,7 +7738,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -6702,72 +7748,232 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Planeter och liv i andra solsystem</t>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara hur exoplaneter upptäcks och vad som krävs för liv, och granska rymdnyheter.</t>
+          <t>Eleven kan förklara jordens strålningsbalans och växthuseffekten och argumentera om klimatförändringar med belägg.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver exoplaneter och livets villkor. C: förklarar metoderna och beboeliga zonen. A: bedömer hur säkra slutsatserna är.</t>
+          <t>E: beskriver växthuseffekten och ger exempel på klimatpåverkan. C: förklarar strålningsbalansen och skillnaden mellan naturlig och förstärkt effekt. A: bedömer klimatmodeller och åtgärder med belägg från flera källor.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Universummodell</t>
+          <t>Strålningsbalansmodell</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Mars och livet; Drake-ekvationen; SETI</t>
+          <t>Istider och klimatets historia; Ozonskiktet; Havens roll i klimatet</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Universum</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
+          <t>Universums uppkomst och uppbyggnad</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Eleven kan beskriva universums uppbyggnad och utveckling och förklara hur modellerna vuxit fram.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>E: beskriver solsystem, galaxer och big bang. C: förklarar bevisen för ett expanderande universum. A: resonerar om modellernas styrkor, begränsningar och föränderlighet.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Universummodell</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Svarta hål; Rymdteleskop; Rymdfärder</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Planeter och liv i andra solsystem</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Eleven kan förklara hur exoplaneter upptäcks och vad som krävs för liv, och granska rymdnyheter.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>E: beskriver exoplaneter och livets villkor. C: förklarar metoderna och beboeliga zonen. A: bedömer hur säkra slutsatserna är.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Universummodell</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Mars och livet; Drake-ekvationen; SETI</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>Repetition inför nationella proven</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Eleven kan koppla ihop partikelmodell, energi, krafter, elektricitet, ljus, ljud och strålning och genomföra och granska undersökningar.</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Materia, energi och krafter</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Eleven kan koppla ihop partikelmodell, energi, krafter och rörelse i nya sammanhang.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>E: använder begreppen i enkla sammanhang. C: kopplar ihop begrepp och förklarar samband. A: använder flera modeller i nya situationer och motiverar.</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Samlad repetition</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Gamla nationella prov; Provstrategier; Begreppskartor</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Gamla nationella prov; Begreppskartor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Elektricitet, ljus, ljud, strålning och universum</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Eleven kan koppla ihop elektricitet, magnetism, ljus, ljud, strålning, klimat och universum i nya sammanhang.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>E: använder begreppen i enkla sammanhang. C: kopplar ihop begrepp och förklarar samband. A: använder flera modeller i nya situationer och motiverar.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Samlad repetition</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Gamla nationella prov</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Undersökningar, källor och argument</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Eleven kan genomföra och värdera undersökningar, granska information och argumentera i frågor om energi, teknik och miljö.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>E: använder begreppen i enkla sammanhang. C: kopplar ihop begrepp och förklarar samband. A: väger källor och argument mot varandra och motiverar.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Samlad repetition</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Gamla nationella prov; Provstrategier</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6778,7 +7984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6905,12 +8111,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ljus och ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Vågor som bär information: hur ljus och ljud uppstår, breder ut sig, reflekteras och registreras.</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts, och hur vi ser färger och bilder.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -6923,12 +8129,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Strålning, väder och klimat</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Strålning från atomkärnor och från solen: användning, risker och hur strålningsbalansen styr klimatet.</t>
+          <t>Hur ljud uppstår, breder ut sig och registreras, och hur vi hör.</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -6941,20 +8147,56 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Universum och helheten</t>
+          <t>Strålning, väder och klimat</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Från solsystemet till universum och sökandet efter liv på andra planeter, med repetition inför de nationella proven.</t>
+          <t>Strålning från atomkärnor och från solen: användning, risker och hur strålningsbalansen styr klimatet.</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Universum</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Från solsystemet till universum och sökandet efter liv på andra planeter.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Repetition inför nationella proven</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Binder ihop fysikens begrepp och modeller, undersökningar och argumentation inför de nationella proven.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6965,7 +8207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7336,22 +8578,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ljus: utbredning, reflektion och brytning</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Reflektion och brytning med ljuslåda</t>
+          <t>Reflektion med ljuslåda</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Hur beter sig ljus vid spegel och i vatten?</t>
+          <t>Hur beter sig ljus när det reflekteras i en spegel?</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Eleverna riktar en ljusstråle mot spegel och vattenbehållare, mäter vinklarna och jämför med reflektionslagen.</t>
+          <t>Eleverna riktar en ljusstråle mot en plan spegel, mäter infalls- och reflektionsvinkel och jämför med reflektionslagen.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -7368,27 +8610,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Hur påverkar längden tonhöjden?</t>
+          <t>Brytning i vatten</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras?</t>
+          <t>Hur bryts ljus när det går från luft till vatten eller glas?</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app.</t>
+          <t>Eleverna riktar en ljusstråle mot en halvcylinder av plast eller en vattenbehållare, mäter infalls- och brytningsvinkel och ritar strålgången.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
+          <t>Titta aldrig in i en laserstråle. Torka upp vatten.</t>
         </is>
       </c>
     </row>
@@ -7400,27 +8642,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Strålning: användning och risker</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Vad stoppar UV-strålning?</t>
+          <t>Hur snabbt går ljudet?</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Vilka material och solskyddsfaktorer skyddar mot UV-strålning?</t>
+          <t>Hur kan ljudets hastighet mätas?</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Eleverna använder UV-känsliga pärlor under UV-lampa eller solljus, täcker med olika material och solkräm och jämför färgförändringen.</t>
+          <t>Eleverna mäter tid för eko över en känd sträcka eller med två mikrofoner och en app, och beräknar v = s/t.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Titta inte rakt in i UV-lampan. Använd solkräm enligt märkning och tvätta händerna.</t>
+          <t>Skydda hörseln: inga höga smällar. Håll avstånd vid utomhusmätning.</t>
         </is>
       </c>
     </row>
@@ -7432,27 +8674,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Strålningsbalans, växthuseffekt och klimat</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Hur påverkar ytans färg uppvärmningen?</t>
+          <t>Hur påverkar längden tonhöjden?</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Hur påverkar ytans färg temperaturen när den belyses?</t>
+          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras?</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Eleverna belyser svarta, vita och silverfärgade ytor med lampa och mäter temperaturen över tid. De kopplar till albedo och klimat.</t>
+          <t>Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden, eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Lampan blir varm. Rör inte lampa eller glödande delar.</t>
+          <t>Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
         </is>
       </c>
     </row>
@@ -7464,27 +8706,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Universums uppkomst och uppbyggnad</t>
+          <t>Strålning: användning och risker</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Solsystemet i skala</t>
+          <t>Vad stoppar UV-strålning?</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Hur stort är solsystemet jämfört med planeterna?</t>
+          <t>Vilka material och solskyddsfaktorer skyddar mot UV-strålning?</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Eleverna bygger en skalmodell med beräknade avstånd (t.ex. 1 m = 1 AU) och diskuterar vad modellen visar och inte visar.</t>
+          <t>Eleverna använder UV-känsliga pärlor under UV-lampa eller solljus, täcker med olika material och solkräm och jämför färgförändringen.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Inga särskilda risker.</t>
+          <t>Titta inte rakt in i UV-lampan. Använd solkräm enligt märkning och tvätta händerna.</t>
         </is>
       </c>
     </row>
@@ -7496,32 +8738,96 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>Strålningsbalans, växthuseffekt och klimat</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Hur påverkar ytans färg uppvärmningen?</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Hur påverkar ytans färg temperaturen när den belyses?</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Eleverna belyser svarta, vita och silverfärgade ytor med lampa och mäter temperaturen över tid. De kopplar till albedo och klimat.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Lampan blir varm. Rör inte lampa eller glödande delar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Universums uppkomst och uppbyggnad</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Solsystemet i skala</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Hur stort är solsystemet jämfört med planeterna?</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Eleverna bygger en skalmodell med beräknade avstånd (t.ex. 1 m = 1 AU) och diskuterar vad modellen visar och inte visar.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Inga särskilda risker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>Planeter och liv i andra solsystem</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Transitmetoden: hur upptäcks planeter?</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Hur ändras ljusstyrkan när en planet passerar framför sin stjärna?</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Eleverna låter en liten boll kretsa framför en lampa och mäter ljusstyrkan med app. De ritar ljuskurvan och kopplar till planetens storlek.</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Lampan blir varm. Tänd bara när det behövs.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7584,7 +8890,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -7599,7 +8905,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -7644,7 +8950,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -7659,7 +8965,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -7674,7 +8980,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -7689,7 +8995,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -7719,7 +9025,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -7764,7 +9070,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -7779,7 +9085,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -7824,7 +9130,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20">
@@ -7839,7 +9145,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21">
@@ -7899,7 +9205,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25">
@@ -7914,7 +9220,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
@@ -7929,7 +9235,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fysik: ljud före ljus (ljus leder över till strålning)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017mqJrSEX6tzqa8YfkctM6P
</commit_message>
<xml_diff>
--- a/planering/fysik-planering.xlsx
+++ b/planering/fysik-planering.xlsx
@@ -3805,7 +3805,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -3825,17 +3825,17 @@
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Ljuskällor och ljusets utbredning</t>
+          <t>Vibrationer och ljudkällor</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>Ljuskällor, rätlinjig utbredning, skuggor, ljusets hastighet och ljusår; hur vi ser.</t>
+          <t>Hur ljud uppstår; ljudkällor och vibrerande föremål.</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>ljuskälla, ljusstråle, skugga, ljushastighet, ljusår</t>
+          <t>vibration, ljudkälla, svängning</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K71" s="4" t="inlineStr">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3880,17 +3880,17 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Reflektion</t>
+          <t>Ljudets utbredning</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Reflektionslagen; plana speglar; spridd reflektion.</t>
+          <t>Ljud i luft, vätskor och fasta ämnen men inte i vakuum; ljudets hastighet.</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>reflektion, spegel, infallsvinkel, reflektionsvinkel</t>
+          <t>medium, ljudhastighet, vakuum</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -3935,27 +3935,27 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Färg och ytor</t>
+          <t>Eko och ljudisolering</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Hur föremål får färg: ljus som absorberas och reflekteras; vitt, svart och färgat ljus.</t>
+          <t>Reflektion och absorption av ljud; eko, efterklang och ljudisolering.</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>absorption, reflektion, färg, spektrum</t>
+          <t>eko, absorption, ljudisolering</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället; Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+          <t>Kunskaper om fysiken i naturen och samhället</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
@@ -3990,17 +3990,17 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Labb: Reflektion med ljuslåda</t>
+          <t>Labb: Hur snabbt går ljudet?</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Hur beter sig ljus när det reflekteras i en spegel? Eleverna riktar en ljusstråle mot en plan spegel, mäter infalls- och reflektionsvinkel och jämför med reflektionslagen. Säkerhet: Titta aldrig in i en laserstråle eller starkt ljus. Rikta inte laser mot ansikten.</t>
+          <t>Hur kan ljudets hastighet mätas? Eleverna mäter tid för eko över en känd sträcka eller med två mikrofoner och en app, och beräknar v = s/t. Säkerhet: Skydda hörseln: inga höga smällar. Håll avstånd vid utomhusmätning.</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>infallsvinkel, reflektionsvinkel, reflektionslagen</t>
+          <t>ljudhastighet, sträcka, tid, eko</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Periskop</t>
+          <t>Åska och ljudets hastighet</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Kamouflage och färg</t>
+          <t>Överljud</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr"/>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -4115,7 +4115,7 @@
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Ljusföroreningar</t>
+          <t>Ljud under vatten</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -4150,17 +4150,17 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Brytning</t>
+          <t>Frekvens och amplitud</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Ljus mellan luft, vatten och glas; ljusets hastighet i olika medier; totalreflektion.</t>
+          <t>Tonhöjd och frekvens (Hz), ljudstyrka och amplitud (dB).</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>brytning, medium, normal, totalreflektion</t>
+          <t>frekvens, hertz, amplitud, decibel</t>
         </is>
       </c>
       <c r="I78" s="4" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K78" s="4" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -4205,27 +4205,27 @@
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Linser och optiska instrument</t>
+          <t>Hörsel och hörselskydd</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>Konvexa och konkava linser; ögat, kikare, mikroskop och kamera.</t>
+          <t>Örats funktion; buller och hörselskador; hörselskydd.</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>lins, brännpunkt, bild, förstoring</t>
+          <t>örat, buller, hörselskada, hörselskydd</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället; Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+          <t>Kunskaper om fysiken i naturen och samhället</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -4250,7 +4250,7 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -4260,27 +4260,27 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Färgspridning och spektrum</t>
+          <t>Registrera ljud</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Prisma, regnbåge och ljusets färger.</t>
+          <t>Mikrofon, frekvensanalys och appar; ultraljud och ekolod.</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>prisma, spektrum, regnbåge, färgspridning</t>
+          <t>mikrofon, ultraljud, ekolod, frekvensanalys</t>
         </is>
       </c>
       <c r="I80" s="4" t="inlineStr">
         <is>
-          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
+          <t>Kunskaper om fysiken i naturen och samhället; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -4315,17 +4315,17 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Labb: Brytning i vatten</t>
+          <t>Labb: Hur påverkar längden tonhöjden?</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Hur bryts ljus när det går från luft till vatten eller glas? Eleverna riktar en ljusstråle mot en halvcylinder av plast eller en vattenbehållare, mäter infalls- och brytningsvinkel och ritar strålgången. Säkerhet: Titta aldrig in i en laserstråle. Torka upp vatten.</t>
+          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras? Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden, eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app. Säkerhet: Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>brytningsvinkel, infallsvinkel, medium</t>
+          <t>frekvens, tonhöjd, vibration, app</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljus breder ut sig, reflekteras och bryts</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Fiberoptik</t>
+          <t>Musikinstrument</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Ögats uppbyggnad</t>
+          <t>Dopplereffekten</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr"/>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Optiska instrument i detalj</t>
+          <t>Akustik i klassrummet</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr"/>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -4475,17 +4475,17 @@
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Vibrationer och ljudkällor</t>
+          <t>Ljuskällor och ljusets utbredning</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår; ljudkällor och vibrerande föremål.</t>
+          <t>Ljuskällor, rätlinjig utbredning, skuggor, ljusets hastighet och ljusår; hur vi ser.</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>vibration, ljudkälla, svängning</t>
+          <t>ljuskälla, ljusstråle, skugga, ljushastighet, ljusår</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
@@ -4530,17 +4530,17 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Ljudets utbredning</t>
+          <t>Reflektion</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>Ljud i luft, vätskor och fasta ämnen men inte i vakuum; ljudets hastighet.</t>
+          <t>Reflektionslagen; plana speglar; spridd reflektion.</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>medium, ljudhastighet, vakuum</t>
+          <t>reflektion, spegel, infallsvinkel, reflektionsvinkel</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -4585,27 +4585,27 @@
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Eko och ljudisolering</t>
+          <t>Färg och ytor</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Reflektion och absorption av ljud; eko, efterklang och ljudisolering.</t>
+          <t>Hur föremål får färg: ljus som absorberas och reflekteras; vitt, svart och färgat ljus.</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>eko, absorption, ljudisolering</t>
+          <t>absorption, reflektion, färg, spektrum</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället</t>
+          <t>Kunskaper om fysiken i naturen och samhället; Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -4640,17 +4640,17 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Labb: Hur snabbt går ljudet?</t>
+          <t>Labb: Reflektion med ljuslåda</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>Hur kan ljudets hastighet mätas? Eleverna mäter tid för eko över en känd sträcka eller med två mikrofoner och en app, och beräknar v = s/t. Säkerhet: Skydda hörseln: inga höga smällar. Håll avstånd vid utomhusmätning.</t>
+          <t>Hur beter sig ljus när det reflekteras i en spegel? Eleverna riktar en ljusstråle mot en plan spegel, mäter infalls- och reflektionsvinkel och jämför med reflektionslagen. Säkerhet: Titta aldrig in i en laserstråle eller starkt ljus. Rikta inte laser mot ansikten.</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>ljudhastighet, sträcka, tid, eko</t>
+          <t>infallsvinkel, reflektionsvinkel, reflektionslagen</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K88" s="4" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Åska och ljudets hastighet</t>
+          <t>Periskop</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr"/>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Överljud</t>
+          <t>Kamouflage och färg</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr"/>
@@ -4745,7 +4745,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Ljud under vatten</t>
+          <t>Ljusföroreningar</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -4800,17 +4800,17 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Frekvens och amplitud</t>
+          <t>Brytning</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd och frekvens (Hz), ljudstyrka och amplitud (dB).</t>
+          <t>Ljus mellan luft, vatten och glas; ljusets hastighet i olika medier; totalreflektion.</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>frekvens, hertz, amplitud, decibel</t>
+          <t>brytning, medium, normal, totalreflektion</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -4855,27 +4855,27 @@
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Hörsel och hörselskydd</t>
+          <t>Linser och optiska instrument</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Örats funktion; buller och hörselskador; hörselskydd.</t>
+          <t>Konvexa och konkava linser; ögat, kikare, mikroskop och kamera.</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>örat, buller, hörselskada, hörselskydd</t>
+          <t>lins, brännpunkt, bild, förstoring</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället</t>
+          <t>Kunskaper om fysiken i naturen och samhället; Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -4910,27 +4910,27 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Registrera ljud</t>
+          <t>Färgspridning och spektrum</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Mikrofon, frekvensanalys och appar; ultraljud och ekolod.</t>
+          <t>Prisma, regnbåge och ljusets färger.</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>mikrofon, ultraljud, ekolod, frekvensanalys</t>
+          <t>prisma, spektrum, regnbåge, färgspridning</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>Kunskaper om fysiken i naturen och samhället; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
+          <t>Använda fysikens begrepp och förklaringsmodeller för att beskriva och förklara fysikaliska fenomen</t>
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -4965,17 +4965,17 @@
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Labb: Hur påverkar längden tonhöjden?</t>
+          <t>Labb: Brytning i vatten</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras? Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden, eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app. Säkerhet: Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
+          <t>Hur bryts ljus när det går från luft till vatten eller glas? Eleverna riktar en ljusstråle mot en halvcylinder av plast eller en vattenbehållare, mäter infalls- och brytningsvinkel och ritar strålgången. Säkerhet: Titta aldrig in i en laserstråle. Torka upp vatten.</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>frekvens, tonhöjd, vibration, app</t>
+          <t>brytningsvinkel, infallsvinkel, medium</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
-          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljud uppstår, breder ut sig och kan registreras på olika sätt</t>
+          <t>Observationer och experiment (analoga och digitala verktyg): undersökningsbara frågor, planering, utförande, värdering och dokumentation; Hur ljus breder ut sig, reflekteras och bryts</t>
         </is>
       </c>
       <c r="K95" s="4" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Musikinstrument</t>
+          <t>Fiberoptik</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr"/>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Dopplereffekten</t>
+          <t>Ögats uppbyggnad</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr"/>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Akustik i klassrummet</t>
+          <t>Optiska instrument i detalj</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -7538,7 +7538,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -7548,27 +7548,27 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara och rita hur ljus breder ut sig och reflekteras och förklara skuggor, speglar och färg.</t>
+          <t>Eleven kan förklara att ljud är vibrationer som breder ut sig i ett medium och beräkna ljudets hastighet.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver ljusets utbredning och ger exempel på reflektion. C: ritar strålgångar och förklarar skuggor och speglar. A: förklarar och förutsäger reflektion och hur ytor ger färg.</t>
+          <t>E: beskriver att ljud är vibrationer och ger exempel. C: förklarar utbredning i olika medier och beräknar hastighet. A: resonerar om mätvärden och om hur ljud reflekteras och absorberas.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Ljusstrålemodell</t>
+          <t>Vågmodell</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Periskop; Kamouflage och färg; Ljusföroreningar</t>
+          <t>Åska och ljudets hastighet; Överljud; Ljud under vatten</t>
         </is>
       </c>
     </row>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -7588,27 +7588,27 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara och rita brytning av ljus och hur linser och optiska instrument fungerar.</t>
+          <t>Eleven kan förklara frekvens och amplitud, hur hörseln fungerar och hur ljud registreras.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver brytning och ger exempel. C: ritar strålgångar genom linser och förklarar prismat. A: förklarar och förutsäger brytning och färgspridning.</t>
+          <t>E: beskriver tonhöjd, ljudstyrka och hörselskydd. C: förklarar frekvens, amplitud och örats funktion. A: resonerar om mätvärden, hörselskador och registrering med digitala verktyg.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Ljusstrålemodell</t>
+          <t>Vågmodell</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Fiberoptik; Ögats uppbyggnad; Optiska instrument i detalj</t>
+          <t>Musikinstrument; Dopplereffekten; Akustik i klassrummet</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -7628,27 +7628,27 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara att ljud är vibrationer som breder ut sig i ett medium och beräkna ljudets hastighet.</t>
+          <t>Eleven kan förklara och rita hur ljus breder ut sig och reflekteras och förklara skuggor, speglar och färg.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver att ljud är vibrationer och ger exempel. C: förklarar utbredning i olika medier och beräknar hastighet. A: resonerar om mätvärden och om hur ljud reflekteras och absorberas.</t>
+          <t>E: beskriver ljusets utbredning och ger exempel på reflektion. C: ritar strålgångar och förklarar skuggor och speglar. A: förklarar och förutsäger reflektion och hur ytor ger färg.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Vågmodell</t>
+          <t>Ljusstrålemodell</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Åska och ljudets hastighet; Överljud; Ljud under vatten</t>
+          <t>Periskop; Kamouflage och färg; Ljusföroreningar</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -7668,27 +7668,27 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Eleven kan förklara frekvens och amplitud, hur hörseln fungerar och hur ljud registreras.</t>
+          <t>Eleven kan förklara och rita brytning av ljus och hur linser och optiska instrument fungerar.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>E: beskriver tonhöjd, ljudstyrka och hörselskydd. C: förklarar frekvens, amplitud och örats funktion. A: resonerar om mätvärden, hörselskador och registrering med digitala verktyg.</t>
+          <t>E: beskriver brytning och ger exempel. C: ritar strålgångar genom linser och förklarar prismat. A: förklarar och förutsäger brytning och färgspridning.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Vågmodell</t>
+          <t>Ljusstrålemodell</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Musikinstrument; Dopplereffekten; Akustik i klassrummet</t>
+          <t>Fiberoptik; Ögats uppbyggnad; Optiska instrument i detalj</t>
         </is>
       </c>
     </row>
@@ -8111,12 +8111,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ljus</t>
+          <t>Ljud</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Hur ljus breder ut sig, reflekteras och bryts, och hur vi ser färger och bilder.</t>
+          <t>Hur ljud uppstår, breder ut sig och registreras, och hur vi hör.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -8129,12 +8129,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Ljud</t>
+          <t>Ljus</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår, breder ut sig och registreras, och hur vi hör.</t>
+          <t>Hur ljus breder ut sig, reflekteras och bryts, och hur vi ser färger och bilder.</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -8578,27 +8578,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ljusets utbredning och reflektion</t>
+          <t>Hur ljud uppstår och breder ut sig</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Reflektion med ljuslåda</t>
+          <t>Hur snabbt går ljudet?</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Hur beter sig ljus när det reflekteras i en spegel?</t>
+          <t>Hur kan ljudets hastighet mätas?</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Eleverna riktar en ljusstråle mot en plan spegel, mäter infalls- och reflektionsvinkel och jämför med reflektionslagen.</t>
+          <t>Eleverna mäter tid för eko över en känd sträcka eller med två mikrofoner och en app, och beräknar v = s/t.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Titta aldrig in i en laserstråle eller starkt ljus. Rikta inte laser mot ansikten.</t>
+          <t>Skydda hörseln: inga höga smällar. Håll avstånd vid utomhusmätning.</t>
         </is>
       </c>
     </row>
@@ -8610,27 +8610,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Brytning, linser och färger</t>
+          <t>Tonhöjd, ljudstyrka och hörsel</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Brytning i vatten</t>
+          <t>Hur påverkar längden tonhöjden?</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Hur bryts ljus när det går från luft till vatten eller glas?</t>
+          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras?</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Eleverna riktar en ljusstråle mot en halvcylinder av plast eller en vattenbehållare, mäter infalls- och brytningsvinkel och ritar strålgången.</t>
+          <t>Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden, eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Titta aldrig in i en laserstråle. Torka upp vatten.</t>
+          <t>Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
         </is>
       </c>
     </row>
@@ -8642,27 +8642,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Hur ljud uppstår och breder ut sig</t>
+          <t>Ljusets utbredning och reflektion</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Hur snabbt går ljudet?</t>
+          <t>Reflektion med ljuslåda</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Hur kan ljudets hastighet mätas?</t>
+          <t>Hur beter sig ljus när det reflekteras i en spegel?</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Eleverna mäter tid för eko över en känd sträcka eller med två mikrofoner och en app, och beräknar v = s/t.</t>
+          <t>Eleverna riktar en ljusstråle mot en plan spegel, mäter infalls- och reflektionsvinkel och jämför med reflektionslagen.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Skydda hörseln: inga höga smällar. Håll avstånd vid utomhusmätning.</t>
+          <t>Titta aldrig in i en laserstråle eller starkt ljus. Rikta inte laser mot ansikten.</t>
         </is>
       </c>
     </row>
@@ -8674,27 +8674,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Tonhöjd, ljudstyrka och hörsel</t>
+          <t>Brytning, linser och färger</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Hur påverkar längden tonhöjden?</t>
+          <t>Brytning i vatten</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Hur ändras tonhöjden när längden på ett vibrerande föremål ändras?</t>
+          <t>Hur bryts ljus när det går från luft till vatten eller glas?</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Eleverna fäster en linjal vid bordskanten och varierar den vibrerande längden, eller fyller flaskor med olika vattennivåer. Frekvensen mäts med en app.</t>
+          <t>Eleverna riktar en ljusstråle mot en halvcylinder av plast eller en vattenbehållare, mäter infalls- och brytningsvinkel och ritar strålgången.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Skydda hörseln: ingen hög ljudnivå. Använd inte vassa föremål.</t>
+          <t>Titta aldrig in i en laserstråle. Torka upp vatten.</t>
         </is>
       </c>
     </row>

</xml_diff>